<commit_message>
universe-1000: fix unified universe portfolio logic, short from top-1000 non-long pool
</commit_message>
<xml_diff>
--- a/Output/130_30_Backtest_Table.xlsx
+++ b/Output/130_30_Backtest_Table.xlsx
@@ -685,12 +685,12 @@
       </c>
       <c r="B6" s="12" t="inlineStr">
         <is>
-          <t>1976-04-01 to 2024-12-01</t>
+          <t>1976-02-01 to 2024-12-01</t>
         </is>
       </c>
       <c r="C6" s="12" t="inlineStr">
         <is>
-          <t>1976-04-01 to 2024-12-01</t>
+          <t>1976-02-01 to 2024-12-01</t>
         </is>
       </c>
       <c r="D6" s="12" t="inlineStr">
@@ -700,7 +700,7 @@
       </c>
       <c r="E6" s="12" t="inlineStr">
         <is>
-          <t>1976-04-01 to 2024-12-01</t>
+          <t>1976-02-01 to 2024-12-01</t>
         </is>
       </c>
       <c r="F6" s="12" t="inlineStr">
@@ -710,7 +710,7 @@
       </c>
       <c r="G6" s="13" t="inlineStr">
         <is>
-          <t>1976-04-01 to 2024-12-01</t>
+          <t>1976-02-01 to 2024-12-01</t>
         </is>
       </c>
     </row>
@@ -721,22 +721,22 @@
         </is>
       </c>
       <c r="B7" s="15" t="n">
-        <v>585</v>
+        <v>587</v>
       </c>
       <c r="C7" s="15" t="n">
-        <v>585</v>
+        <v>587</v>
       </c>
       <c r="D7" s="15" t="n">
         <v>606</v>
       </c>
       <c r="E7" s="15" t="n">
-        <v>585</v>
+        <v>587</v>
       </c>
       <c r="F7" s="15" t="n">
         <v>606</v>
       </c>
       <c r="G7" s="16" t="n">
-        <v>585</v>
+        <v>587</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
@@ -754,32 +754,32 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>16.71%</t>
+          <t>18.01%</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>15.90%</t>
+          <t>15.60%</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
-          <t>15.47%</t>
+          <t>16.24%</t>
         </is>
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>-11.08%</t>
+          <t>-10.48%</t>
         </is>
       </c>
       <c r="F9" s="12" t="inlineStr">
         <is>
-          <t>14.39%</t>
+          <t>14.07%</t>
         </is>
       </c>
       <c r="G9" s="13" t="inlineStr">
         <is>
-          <t>-9.92%</t>
+          <t>-9.68%</t>
         </is>
       </c>
     </row>
@@ -791,32 +791,32 @@
       </c>
       <c r="B10" s="18" t="inlineStr">
         <is>
-          <t>16.59%</t>
+          <t>17.90%</t>
         </is>
       </c>
       <c r="C10" s="18" t="inlineStr">
         <is>
-          <t>15.77%</t>
+          <t>15.16%</t>
         </is>
       </c>
       <c r="D10" s="18" t="inlineStr">
         <is>
-          <t>15.07%</t>
+          <t>15.67%</t>
         </is>
       </c>
       <c r="E10" s="18" t="inlineStr">
         <is>
-          <t>-11.97%</t>
+          <t>-12.02%</t>
         </is>
       </c>
       <c r="F10" s="18" t="inlineStr">
         <is>
-          <t>14.00%</t>
+          <t>13.41%</t>
         </is>
       </c>
       <c r="G10" s="19" t="inlineStr">
         <is>
-          <t>-10.80%</t>
+          <t>-10.96%</t>
         </is>
       </c>
     </row>
@@ -828,32 +828,32 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>15.91%</t>
+          <t>16.91%</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>15.31%</t>
+          <t>16.80%</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
-          <t>16.45%</t>
+          <t>17.87%</t>
         </is>
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>17.96%</t>
+          <t>21.34%</t>
         </is>
       </c>
       <c r="F11" s="12" t="inlineStr">
         <is>
-          <t>15.63%</t>
+          <t>16.86%</t>
         </is>
       </c>
       <c r="G11" s="13" t="inlineStr">
         <is>
-          <t>17.11%</t>
+          <t>19.43%</t>
         </is>
       </c>
     </row>
@@ -865,32 +865,32 @@
       </c>
       <c r="B12" s="18" t="inlineStr">
         <is>
-          <t>1.05</t>
+          <t>1.07</t>
         </is>
       </c>
       <c r="C12" s="18" t="inlineStr">
         <is>
-          <t>1.04</t>
+          <t>0.93</t>
         </is>
       </c>
       <c r="D12" s="18" t="inlineStr">
         <is>
-          <t>0.94</t>
+          <t>0.91</t>
         </is>
       </c>
       <c r="E12" s="18" t="inlineStr">
         <is>
-          <t>-0.62</t>
+          <t>-0.49</t>
         </is>
       </c>
       <c r="F12" s="18" t="inlineStr">
         <is>
-          <t>0.92</t>
+          <t>0.83</t>
         </is>
       </c>
       <c r="G12" s="19" t="inlineStr">
         <is>
-          <t>-0.58</t>
+          <t>-0.50</t>
         </is>
       </c>
     </row>
@@ -902,27 +902,27 @@
       </c>
       <c r="B13" s="21" t="inlineStr">
         <is>
-          <t>-37.06%</t>
+          <t>-37.98%</t>
         </is>
       </c>
       <c r="C13" s="21" t="inlineStr">
         <is>
-          <t>-35.68%</t>
+          <t>-46.48%</t>
         </is>
       </c>
       <c r="D13" s="21" t="inlineStr">
         <is>
-          <t>-44.81%</t>
+          <t>-46.06%</t>
         </is>
       </c>
       <c r="E13" s="21" t="inlineStr">
         <is>
-          <t>-99.82%</t>
+          <t>-99.83%</t>
         </is>
       </c>
       <c r="F13" s="21" t="inlineStr">
         <is>
-          <t>-40.80%</t>
+          <t>-47.56%</t>
         </is>
       </c>
       <c r="G13" s="22" t="inlineStr">
@@ -946,32 +946,32 @@
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>1.80</t>
+          <t>1.82</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>1.81</t>
+          <t>1.59</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
         <is>
-          <t>1.59</t>
+          <t>1.51</t>
         </is>
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>-0.81</t>
+          <t>-0.66</t>
         </is>
       </c>
       <c r="F15" s="12" t="inlineStr">
         <is>
-          <t>1.54</t>
+          <t>1.37</t>
         </is>
       </c>
       <c r="G15" s="13" t="inlineStr">
         <is>
-          <t>-0.76</t>
+          <t>-0.67</t>
         </is>
       </c>
     </row>
@@ -983,12 +983,12 @@
       </c>
       <c r="B16" s="18" t="inlineStr">
         <is>
-          <t>0.45</t>
+          <t>0.47</t>
         </is>
       </c>
       <c r="C16" s="18" t="inlineStr">
         <is>
-          <t>0.45</t>
+          <t>0.34</t>
         </is>
       </c>
       <c r="D16" s="18" t="inlineStr">
@@ -998,12 +998,12 @@
       </c>
       <c r="E16" s="18" t="inlineStr">
         <is>
-          <t>-0.11</t>
+          <t>-0.10</t>
         </is>
       </c>
       <c r="F16" s="18" t="inlineStr">
         <is>
-          <t>0.35</t>
+          <t>0.30</t>
         </is>
       </c>
       <c r="G16" s="19" t="inlineStr">
@@ -1020,32 +1020,32 @@
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>-23.35%</t>
+          <t>-24.38%</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>-19.78%</t>
+          <t>-21.04%</t>
         </is>
       </c>
       <c r="D17" s="12" t="inlineStr">
         <is>
-          <t>-23.65%</t>
+          <t>-25.64%</t>
         </is>
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>-19.13%</t>
+          <t>-26.81%</t>
         </is>
       </c>
       <c r="F17" s="12" t="inlineStr">
         <is>
-          <t>-20.60%</t>
+          <t>-22.16%</t>
         </is>
       </c>
       <c r="G17" s="13" t="inlineStr">
         <is>
-          <t>-18.67%</t>
+          <t>-25.01%</t>
         </is>
       </c>
     </row>
@@ -1057,32 +1057,32 @@
       </c>
       <c r="B18" s="18" t="inlineStr">
         <is>
-          <t>64.4%</t>
+          <t>64.9%</t>
         </is>
       </c>
       <c r="C18" s="18" t="inlineStr">
         <is>
-          <t>64.4%</t>
+          <t>62.0%</t>
         </is>
       </c>
       <c r="D18" s="18" t="inlineStr">
         <is>
-          <t>62.5%</t>
+          <t>62.4%</t>
         </is>
       </c>
       <c r="E18" s="18" t="inlineStr">
         <is>
-          <t>39.1%</t>
+          <t>40.4%</t>
         </is>
       </c>
       <c r="F18" s="18" t="inlineStr">
         <is>
-          <t>64.4%</t>
+          <t>61.9%</t>
         </is>
       </c>
       <c r="G18" s="19" t="inlineStr">
         <is>
-          <t>38.5%</t>
+          <t>39.7%</t>
         </is>
       </c>
     </row>
@@ -1094,32 +1094,32 @@
       </c>
       <c r="B19" s="12" t="inlineStr">
         <is>
-          <t>-0.38</t>
+          <t>-0.39</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
+          <t>-0.08</t>
+        </is>
+      </c>
+      <c r="D19" s="12" t="inlineStr">
+        <is>
+          <t>-0.27</t>
+        </is>
+      </c>
+      <c r="E19" s="12" t="inlineStr">
+        <is>
+          <t>0.61</t>
+        </is>
+      </c>
+      <c r="F19" s="12" t="inlineStr">
+        <is>
           <t>-0.19</t>
         </is>
       </c>
-      <c r="D19" s="12" t="inlineStr">
-        <is>
-          <t>-0.19</t>
-        </is>
-      </c>
-      <c r="E19" s="12" t="inlineStr">
-        <is>
-          <t>0.60</t>
-        </is>
-      </c>
-      <c r="F19" s="12" t="inlineStr">
-        <is>
-          <t>-0.19</t>
-        </is>
-      </c>
       <c r="G19" s="13" t="inlineStr">
         <is>
-          <t>0.51</t>
+          <t>0.54</t>
         </is>
       </c>
     </row>
@@ -1131,32 +1131,32 @@
       </c>
       <c r="B20" s="15" t="inlineStr">
         <is>
-          <t>1.89</t>
+          <t>1.76</t>
         </is>
       </c>
       <c r="C20" s="15" t="inlineStr">
         <is>
-          <t>1.11</t>
+          <t>1.66</t>
         </is>
       </c>
       <c r="D20" s="15" t="inlineStr">
         <is>
-          <t>2.44</t>
+          <t>2.29</t>
         </is>
       </c>
       <c r="E20" s="15" t="inlineStr">
         <is>
-          <t>2.18</t>
+          <t>2.73</t>
         </is>
       </c>
       <c r="F20" s="15" t="inlineStr">
         <is>
-          <t>1.67</t>
+          <t>1.81</t>
         </is>
       </c>
       <c r="G20" s="16" t="inlineStr">
         <is>
-          <t>2.17</t>
+          <t>2.79</t>
         </is>
       </c>
     </row>
@@ -1175,32 +1175,32 @@
       </c>
       <c r="B22" s="12" t="inlineStr">
         <is>
-          <t>7.33</t>
+          <t>7.45</t>
         </is>
       </c>
       <c r="C22" s="12" t="inlineStr">
         <is>
-          <t>7.25</t>
+          <t>6.49</t>
         </is>
       </c>
       <c r="D22" s="12" t="inlineStr">
         <is>
-          <t>6.68</t>
+          <t>6.46</t>
         </is>
       </c>
       <c r="E22" s="12" t="inlineStr">
         <is>
-          <t>-4.31</t>
+          <t>-3.43</t>
         </is>
       </c>
       <c r="F22" s="12" t="inlineStr">
         <is>
-          <t>6.54</t>
+          <t>5.93</t>
         </is>
       </c>
       <c r="G22" s="13" t="inlineStr">
         <is>
-          <t>-4.05</t>
+          <t>-3.48</t>
         </is>
       </c>
     </row>
@@ -1227,17 +1227,17 @@
       </c>
       <c r="E23" s="18" t="inlineStr">
         <is>
+          <t>0.0006</t>
+        </is>
+      </c>
+      <c r="F23" s="18" t="inlineStr">
+        <is>
           <t>0.0000</t>
         </is>
       </c>
-      <c r="F23" s="18" t="inlineStr">
-        <is>
-          <t>0.0000</t>
-        </is>
-      </c>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>0.0001</t>
+          <t>0.0005</t>
         </is>
       </c>
     </row>
@@ -1249,32 +1249,32 @@
       </c>
       <c r="B24" s="21" t="inlineStr">
         <is>
-          <t>[12.24%, 21.18%]</t>
+          <t>[13.27%, 22.75%]</t>
         </is>
       </c>
       <c r="C24" s="21" t="inlineStr">
         <is>
-          <t>[11.60%, 20.19%]</t>
+          <t>[10.89%, 20.31%]</t>
         </is>
       </c>
       <c r="D24" s="21" t="inlineStr">
         <is>
-          <t>[10.93%, 20.00%]</t>
+          <t>[11.31%, 21.17%]</t>
         </is>
       </c>
       <c r="E24" s="21" t="inlineStr">
         <is>
-          <t>[-16.13%, -6.04%]</t>
+          <t>[-16.46%, -4.50%]</t>
         </is>
       </c>
       <c r="F24" s="21" t="inlineStr">
         <is>
-          <t>[10.08%, 18.70%]</t>
+          <t>[9.42%, 18.72%]</t>
         </is>
       </c>
       <c r="G24" s="22" t="inlineStr">
         <is>
-          <t>[-14.73%, -5.12%]</t>
+          <t>[-15.12%, -4.23%]</t>
         </is>
       </c>
     </row>
@@ -1293,32 +1293,32 @@
       </c>
       <c r="B26" s="12" t="inlineStr">
         <is>
-          <t>4.69%</t>
+          <t>5.60%</t>
         </is>
       </c>
       <c r="C26" s="12" t="inlineStr">
         <is>
-          <t>4.67%</t>
+          <t>4.02%</t>
         </is>
       </c>
       <c r="D26" s="12" t="inlineStr">
         <is>
-          <t>3.02%</t>
+          <t>3.22%</t>
         </is>
       </c>
       <c r="E26" s="12" t="inlineStr">
         <is>
-          <t>-1.90%</t>
+          <t>0.16%</t>
         </is>
       </c>
       <c r="F26" s="12" t="inlineStr">
         <is>
-          <t>2.54%</t>
+          <t>1.79%</t>
         </is>
       </c>
       <c r="G26" s="13" t="inlineStr">
         <is>
-          <t>-1.24%</t>
+          <t>-0.02%</t>
         </is>
       </c>
     </row>
@@ -1330,32 +1330,32 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>0.90%</t>
+          <t>1.09%</t>
         </is>
       </c>
       <c r="C27" s="18" t="inlineStr">
         <is>
-          <t>1.23%</t>
+          <t>1.54%</t>
         </is>
       </c>
       <c r="D27" s="18" t="inlineStr">
         <is>
-          <t>0.65%</t>
+          <t>0.86%</t>
         </is>
       </c>
       <c r="E27" s="18" t="inlineStr">
         <is>
-          <t>0.95%</t>
+          <t>1.25%</t>
         </is>
       </c>
       <c r="F27" s="18" t="inlineStr">
         <is>
-          <t>0.88%</t>
+          <t>1.07%</t>
         </is>
       </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>0.98%</t>
+          <t>1.28%</t>
         </is>
       </c>
     </row>
@@ -1367,32 +1367,32 @@
       </c>
       <c r="B28" s="12" t="inlineStr">
         <is>
-          <t>5.23</t>
+          <t>5.14</t>
         </is>
       </c>
       <c r="C28" s="12" t="inlineStr">
         <is>
-          <t>3.80</t>
+          <t>2.60</t>
         </is>
       </c>
       <c r="D28" s="12" t="inlineStr">
         <is>
-          <t>4.61</t>
+          <t>3.73</t>
         </is>
       </c>
       <c r="E28" s="12" t="inlineStr">
         <is>
-          <t>-1.99</t>
+          <t>0.13</t>
         </is>
       </c>
       <c r="F28" s="12" t="inlineStr">
         <is>
-          <t>2.89</t>
+          <t>1.67</t>
         </is>
       </c>
       <c r="G28" s="13" t="inlineStr">
         <is>
-          <t>-1.26</t>
+          <t>-0.01</t>
         </is>
       </c>
     </row>
@@ -1409,27 +1409,27 @@
       </c>
       <c r="C29" s="18" t="inlineStr">
         <is>
-          <t>0.0001</t>
+          <t>0.0092</t>
         </is>
       </c>
       <c r="D29" s="18" t="inlineStr">
         <is>
-          <t>0.0000</t>
+          <t>0.0002</t>
         </is>
       </c>
       <c r="E29" s="18" t="inlineStr">
         <is>
-          <t>0.0467</t>
+          <t>0.8968</t>
         </is>
       </c>
       <c r="F29" s="18" t="inlineStr">
         <is>
-          <t>0.0038</t>
+          <t>0.0950</t>
         </is>
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>0.2059</t>
+          <t>0.9905</t>
         </is>
       </c>
     </row>
@@ -1441,32 +1441,32 @@
       </c>
       <c r="B30" s="12" t="inlineStr">
         <is>
-          <t>[2.93%, 6.44%]</t>
+          <t>[3.46%, 7.73%]</t>
         </is>
       </c>
       <c r="C30" s="12" t="inlineStr">
         <is>
-          <t>[2.26%, 7.07%]</t>
+          <t>[1.00%, 7.05%]</t>
         </is>
       </c>
       <c r="D30" s="12" t="inlineStr">
         <is>
-          <t>[1.74%, 4.30%]</t>
+          <t>[1.53%, 4.92%]</t>
         </is>
       </c>
       <c r="E30" s="12" t="inlineStr">
         <is>
-          <t>[-3.77%, -0.03%]</t>
+          <t>[-2.28%, 2.60%]</t>
         </is>
       </c>
       <c r="F30" s="12" t="inlineStr">
         <is>
-          <t>[0.82%, 4.27%]</t>
+          <t>[-0.31%, 3.89%]</t>
         </is>
       </c>
       <c r="G30" s="13" t="inlineStr">
         <is>
-          <t>[-3.17%, 0.68%]</t>
+          <t>[-2.51%, 2.48%]</t>
         </is>
       </c>
     </row>
@@ -1478,32 +1478,32 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>0.946</t>
+          <t>0.990</t>
         </is>
       </c>
       <c r="C31" s="18" t="inlineStr">
         <is>
-          <t>0.851</t>
+          <t>0.889</t>
         </is>
       </c>
       <c r="D31" s="18" t="inlineStr">
         <is>
-          <t>0.971</t>
+          <t>1.038</t>
         </is>
       </c>
       <c r="E31" s="18" t="inlineStr">
         <is>
-          <t>-1.107</t>
+          <t>-1.279</t>
         </is>
       </c>
       <c r="F31" s="18" t="inlineStr">
         <is>
-          <t>0.899</t>
+          <t>0.951</t>
         </is>
       </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>-1.046</t>
+          <t>-1.161</t>
         </is>
       </c>
     </row>
@@ -1515,32 +1515,32 @@
       </c>
       <c r="B32" s="21" t="inlineStr">
         <is>
-          <t>36.80</t>
+          <t>39.22</t>
         </is>
       </c>
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>28.32</t>
+          <t>19.58</t>
         </is>
       </c>
       <c r="D32" s="21" t="inlineStr">
         <is>
-          <t>38.85</t>
+          <t>37.12</t>
         </is>
       </c>
       <c r="E32" s="21" t="inlineStr">
         <is>
-          <t>-55.97</t>
+          <t>-39.61</t>
         </is>
       </c>
       <c r="F32" s="21" t="inlineStr">
         <is>
-          <t>42.98</t>
+          <t>32.26</t>
         </is>
       </c>
       <c r="G32" s="22" t="inlineStr">
         <is>
-          <t>-39.05</t>
+          <t>-31.25</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
short-mid-caps: confirmed working, short from ranks 501-1000 mid-cap universe
</commit_message>
<xml_diff>
--- a/Output/130_30_Backtest_Table.xlsx
+++ b/Output/130_30_Backtest_Table.xlsx
@@ -754,12 +754,12 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>16.26%</t>
+          <t>16.65%</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>15.04%</t>
+          <t>15.25%</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
@@ -769,7 +769,7 @@
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>-12.82%</t>
+          <t>-11.55%</t>
         </is>
       </c>
       <c r="F9" s="12" t="inlineStr">
@@ -779,7 +779,7 @@
       </c>
       <c r="G9" s="13" t="inlineStr">
         <is>
-          <t>-12.27%</t>
+          <t>-11.57%</t>
         </is>
       </c>
     </row>
@@ -791,12 +791,12 @@
       </c>
       <c r="B10" s="18" t="inlineStr">
         <is>
-          <t>16.14%</t>
+          <t>16.60%</t>
         </is>
       </c>
       <c r="C10" s="18" t="inlineStr">
         <is>
-          <t>14.79%</t>
+          <t>15.05%</t>
         </is>
       </c>
       <c r="D10" s="18" t="inlineStr">
@@ -806,7 +806,7 @@
       </c>
       <c r="E10" s="18" t="inlineStr">
         <is>
-          <t>-14.06%</t>
+          <t>-12.90%</t>
         </is>
       </c>
       <c r="F10" s="18" t="inlineStr">
@@ -816,7 +816,7 @@
       </c>
       <c r="G10" s="19" t="inlineStr">
         <is>
-          <t>-13.47%</t>
+          <t>-12.87%</t>
         </is>
       </c>
     </row>
@@ -828,12 +828,12 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>15.55%</t>
+          <t>15.41%</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>15.31%</t>
+          <t>15.21%</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
@@ -843,7 +843,7 @@
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>21.11%</t>
+          <t>20.99%</t>
         </is>
       </c>
       <c r="F11" s="12" t="inlineStr">
@@ -853,7 +853,7 @@
       </c>
       <c r="G11" s="13" t="inlineStr">
         <is>
-          <t>20.56%</t>
+          <t>20.71%</t>
         </is>
       </c>
     </row>
@@ -865,12 +865,12 @@
       </c>
       <c r="B12" s="18" t="inlineStr">
         <is>
-          <t>1.05</t>
+          <t>1.08</t>
         </is>
       </c>
       <c r="C12" s="18" t="inlineStr">
         <is>
-          <t>0.98</t>
+          <t>1.00</t>
         </is>
       </c>
       <c r="D12" s="18" t="inlineStr">
@@ -880,7 +880,7 @@
       </c>
       <c r="E12" s="18" t="inlineStr">
         <is>
-          <t>-0.61</t>
+          <t>-0.55</t>
         </is>
       </c>
       <c r="F12" s="18" t="inlineStr">
@@ -890,7 +890,7 @@
       </c>
       <c r="G12" s="19" t="inlineStr">
         <is>
-          <t>-0.60</t>
+          <t>-0.56</t>
         </is>
       </c>
     </row>
@@ -902,12 +902,12 @@
       </c>
       <c r="B13" s="21" t="inlineStr">
         <is>
-          <t>-40.28%</t>
+          <t>-40.24%</t>
         </is>
       </c>
       <c r="C13" s="21" t="inlineStr">
         <is>
-          <t>-37.70%</t>
+          <t>-36.75%</t>
         </is>
       </c>
       <c r="D13" s="21" t="inlineStr">
@@ -917,7 +917,7 @@
       </c>
       <c r="E13" s="21" t="inlineStr">
         <is>
-          <t>-99.94%</t>
+          <t>-99.89%</t>
         </is>
       </c>
       <c r="F13" s="21" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="G13" s="22" t="inlineStr">
         <is>
-          <t>-99.92%</t>
+          <t>-99.89%</t>
         </is>
       </c>
     </row>
@@ -946,12 +946,12 @@
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>1.81</t>
+          <t>1.88</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>1.72</t>
+          <t>1.77</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
@@ -961,7 +961,7 @@
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>-0.78</t>
+          <t>-0.73</t>
         </is>
       </c>
       <c r="F15" s="12" t="inlineStr">
@@ -971,7 +971,7 @@
       </c>
       <c r="G15" s="13" t="inlineStr">
         <is>
-          <t>-0.78</t>
+          <t>-0.74</t>
         </is>
       </c>
     </row>
@@ -983,12 +983,12 @@
       </c>
       <c r="B16" s="18" t="inlineStr">
         <is>
-          <t>0.40</t>
+          <t>0.41</t>
         </is>
       </c>
       <c r="C16" s="18" t="inlineStr">
         <is>
-          <t>0.40</t>
+          <t>0.41</t>
         </is>
       </c>
       <c r="D16" s="18" t="inlineStr">
@@ -998,7 +998,7 @@
       </c>
       <c r="E16" s="18" t="inlineStr">
         <is>
-          <t>-0.13</t>
+          <t>-0.12</t>
         </is>
       </c>
       <c r="F16" s="18" t="inlineStr">
@@ -1020,12 +1020,12 @@
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>-22.10%</t>
+          <t>-21.86%</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>-18.25%</t>
+          <t>-18.11%</t>
         </is>
       </c>
       <c r="D17" s="12" t="inlineStr">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>-29.63%</t>
+          <t>-25.98%</t>
         </is>
       </c>
       <c r="F17" s="12" t="inlineStr">
@@ -1045,7 +1045,7 @@
       </c>
       <c r="G17" s="13" t="inlineStr">
         <is>
-          <t>-22.07%</t>
+          <t>-24.11%</t>
         </is>
       </c>
     </row>
@@ -1057,12 +1057,12 @@
       </c>
       <c r="B18" s="18" t="inlineStr">
         <is>
-          <t>62.9%</t>
+          <t>64.6%</t>
         </is>
       </c>
       <c r="C18" s="18" t="inlineStr">
         <is>
-          <t>64.1%</t>
+          <t>64.6%</t>
         </is>
       </c>
       <c r="D18" s="18" t="inlineStr">
@@ -1072,7 +1072,7 @@
       </c>
       <c r="E18" s="18" t="inlineStr">
         <is>
-          <t>39.3%</t>
+          <t>40.0%</t>
         </is>
       </c>
       <c r="F18" s="18" t="inlineStr">
@@ -1094,7 +1094,7 @@
       </c>
       <c r="B19" s="12" t="inlineStr">
         <is>
-          <t>-0.30</t>
+          <t>-0.32</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
@@ -1109,7 +1109,7 @@
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>0.37</t>
+          <t>0.55</t>
         </is>
       </c>
       <c r="F19" s="12" t="inlineStr">
@@ -1131,12 +1131,12 @@
       </c>
       <c r="B20" s="15" t="inlineStr">
         <is>
-          <t>1.65</t>
+          <t>1.67</t>
         </is>
       </c>
       <c r="C20" s="15" t="inlineStr">
         <is>
-          <t>0.89</t>
+          <t>0.88</t>
         </is>
       </c>
       <c r="D20" s="15" t="inlineStr">
@@ -1146,7 +1146,7 @@
       </c>
       <c r="E20" s="15" t="inlineStr">
         <is>
-          <t>3.19</t>
+          <t>2.79</t>
         </is>
       </c>
       <c r="F20" s="15" t="inlineStr">
@@ -1156,7 +1156,7 @@
       </c>
       <c r="G20" s="16" t="inlineStr">
         <is>
-          <t>2.69</t>
+          <t>2.72</t>
         </is>
       </c>
     </row>
@@ -1175,12 +1175,12 @@
       </c>
       <c r="B22" s="12" t="inlineStr">
         <is>
-          <t>7.28</t>
+          <t>7.52</t>
         </is>
       </c>
       <c r="C22" s="12" t="inlineStr">
         <is>
-          <t>6.84</t>
+          <t>6.98</t>
         </is>
       </c>
       <c r="D22" s="12" t="inlineStr">
@@ -1190,7 +1190,7 @@
       </c>
       <c r="E22" s="12" t="inlineStr">
         <is>
-          <t>-4.23</t>
+          <t>-3.83</t>
         </is>
       </c>
       <c r="F22" s="12" t="inlineStr">
@@ -1200,7 +1200,7 @@
       </c>
       <c r="G22" s="13" t="inlineStr">
         <is>
-          <t>-4.16</t>
+          <t>-3.89</t>
         </is>
       </c>
     </row>
@@ -1227,17 +1227,17 @@
       </c>
       <c r="E23" s="18" t="inlineStr">
         <is>
+          <t>0.0001</t>
+        </is>
+      </c>
+      <c r="F23" s="18" t="inlineStr">
+        <is>
           <t>0.0000</t>
         </is>
       </c>
-      <c r="F23" s="18" t="inlineStr">
-        <is>
-          <t>0.0000</t>
-        </is>
-      </c>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>0.0000</t>
+          <t>0.0001</t>
         </is>
       </c>
     </row>
@@ -1249,12 +1249,12 @@
       </c>
       <c r="B24" s="21" t="inlineStr">
         <is>
-          <t>[11.89%, 20.64%]</t>
+          <t>[12.31%, 20.98%]</t>
         </is>
       </c>
       <c r="C24" s="21" t="inlineStr">
         <is>
-          <t>[10.73%, 19.34%]</t>
+          <t>[10.97%, 19.53%]</t>
         </is>
       </c>
       <c r="D24" s="21" t="inlineStr">
@@ -1264,7 +1264,7 @@
       </c>
       <c r="E24" s="21" t="inlineStr">
         <is>
-          <t>[-18.76%, -6.88%]</t>
+          <t>[-17.45%, -5.64%]</t>
         </is>
       </c>
       <c r="F24" s="21" t="inlineStr">
@@ -1274,7 +1274,7 @@
       </c>
       <c r="G24" s="22" t="inlineStr">
         <is>
-          <t>[-18.06%, -6.49%]</t>
+          <t>[-17.40%, -5.74%]</t>
         </is>
       </c>
     </row>
@@ -1293,12 +1293,12 @@
       </c>
       <c r="B26" s="12" t="inlineStr">
         <is>
-          <t>4.48%</t>
+          <t>4.91%</t>
         </is>
       </c>
       <c r="C26" s="12" t="inlineStr">
         <is>
-          <t>4.16%</t>
+          <t>4.42%</t>
         </is>
       </c>
       <c r="D26" s="12" t="inlineStr">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="E26" s="12" t="inlineStr">
         <is>
-          <t>-2.76%</t>
+          <t>-1.33%</t>
         </is>
       </c>
       <c r="F26" s="12" t="inlineStr">
@@ -1318,7 +1318,7 @@
       </c>
       <c r="G26" s="13" t="inlineStr">
         <is>
-          <t>-2.32%</t>
+          <t>-1.47%</t>
         </is>
       </c>
     </row>
@@ -1330,12 +1330,12 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>0.92%</t>
+          <t>0.89%</t>
         </is>
       </c>
       <c r="C27" s="18" t="inlineStr">
         <is>
-          <t>1.33%</t>
+          <t>1.32%</t>
         </is>
       </c>
       <c r="D27" s="18" t="inlineStr">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="E27" s="18" t="inlineStr">
         <is>
-          <t>1.68%</t>
+          <t>1.40%</t>
         </is>
       </c>
       <c r="F27" s="18" t="inlineStr">
@@ -1355,7 +1355,7 @@
       </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>1.43%</t>
+          <t>1.36%</t>
         </is>
       </c>
     </row>
@@ -1367,12 +1367,12 @@
       </c>
       <c r="B28" s="12" t="inlineStr">
         <is>
-          <t>4.88</t>
+          <t>5.55</t>
         </is>
       </c>
       <c r="C28" s="12" t="inlineStr">
         <is>
-          <t>3.13</t>
+          <t>3.35</t>
         </is>
       </c>
       <c r="D28" s="12" t="inlineStr">
@@ -1382,7 +1382,7 @@
       </c>
       <c r="E28" s="12" t="inlineStr">
         <is>
-          <t>-1.64</t>
+          <t>-0.95</t>
         </is>
       </c>
       <c r="F28" s="12" t="inlineStr">
@@ -1392,7 +1392,7 @@
       </c>
       <c r="G28" s="13" t="inlineStr">
         <is>
-          <t>-1.62</t>
+          <t>-1.08</t>
         </is>
       </c>
     </row>
@@ -1409,7 +1409,7 @@
       </c>
       <c r="C29" s="18" t="inlineStr">
         <is>
-          <t>0.0017</t>
+          <t>0.0008</t>
         </is>
       </c>
       <c r="D29" s="18" t="inlineStr">
@@ -1419,7 +1419,7 @@
       </c>
       <c r="E29" s="18" t="inlineStr">
         <is>
-          <t>0.1003</t>
+          <t>0.3428</t>
         </is>
       </c>
       <c r="F29" s="18" t="inlineStr">
@@ -1429,7 +1429,7 @@
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>0.1056</t>
+          <t>0.2814</t>
         </is>
       </c>
     </row>
@@ -1441,12 +1441,12 @@
       </c>
       <c r="B30" s="12" t="inlineStr">
         <is>
-          <t>[2.68%, 6.28%]</t>
+          <t>[3.18%, 6.65%]</t>
         </is>
       </c>
       <c r="C30" s="12" t="inlineStr">
         <is>
-          <t>[1.56%, 6.76%]</t>
+          <t>[1.83%, 7.00%]</t>
         </is>
       </c>
       <c r="D30" s="12" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="E30" s="12" t="inlineStr">
         <is>
-          <t>[-6.05%, 0.53%]</t>
+          <t>[-4.08%, 1.42%]</t>
         </is>
       </c>
       <c r="F30" s="12" t="inlineStr">
@@ -1466,7 +1466,7 @@
       </c>
       <c r="G30" s="13" t="inlineStr">
         <is>
-          <t>[-5.13%, 0.49%]</t>
+          <t>[-4.13%, 1.20%]</t>
         </is>
       </c>
     </row>
@@ -1478,12 +1478,12 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>0.916</t>
+          <t>0.910</t>
         </is>
       </c>
       <c r="C31" s="18" t="inlineStr">
         <is>
-          <t>0.807</t>
+          <t>0.801</t>
         </is>
       </c>
       <c r="D31" s="18" t="inlineStr">
@@ -1493,7 +1493,7 @@
       </c>
       <c r="E31" s="18" t="inlineStr">
         <is>
-          <t>-1.210</t>
+          <t>-1.229</t>
         </is>
       </c>
       <c r="F31" s="18" t="inlineStr">
@@ -1503,7 +1503,7 @@
       </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>-1.197</t>
+          <t>-1.215</t>
         </is>
       </c>
     </row>
@@ -1515,12 +1515,12 @@
       </c>
       <c r="B32" s="21" t="inlineStr">
         <is>
-          <t>34.35</t>
+          <t>34.24</t>
         </is>
       </c>
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>25.13</t>
+          <t>24.97</t>
         </is>
       </c>
       <c r="D32" s="21" t="inlineStr">
@@ -1530,7 +1530,7 @@
       </c>
       <c r="E32" s="21" t="inlineStr">
         <is>
-          <t>-37.04</t>
+          <t>-37.69</t>
         </is>
       </c>
       <c r="F32" s="21" t="inlineStr">
@@ -1540,7 +1540,7 @@
       </c>
       <c r="G32" s="22" t="inlineStr">
         <is>
-          <t>-36.80</t>
+          <t>-37.61</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
switched structure to market neutral
</commit_message>
<xml_diff>
--- a/Output/130_30_Backtest_Table.xlsx
+++ b/Output/130_30_Backtest_Table.xlsx
@@ -628,7 +628,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Composite z-score: Shareholder Yield + Gross Profitability + ROIC  |  130% long top-100 / 30% short bottom-100 (S&amp;P 500 proxy)  |  Quarterly rebalancing, ±5 pp sector neutrality</t>
+          <t>Composite z-score: Shareholder Yield + Gross Profitability + ROIC  |  130% long top-100 / 30% short bottom-100 (Russell 1000 proxy, top 1000 by mktcap)  |  Monthly rebalancing, ±5 pp sector neutrality</t>
         </is>
       </c>
     </row>
@@ -754,22 +754,22 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>18.01%</t>
+          <t>17.95%</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>15.60%</t>
+          <t>15.57%</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
-          <t>16.24%</t>
+          <t>16.18%</t>
         </is>
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>-10.48%</t>
+          <t>-10.43%</t>
         </is>
       </c>
       <c r="F9" s="12" t="inlineStr">
@@ -779,7 +779,7 @@
       </c>
       <c r="G9" s="13" t="inlineStr">
         <is>
-          <t>-9.68%</t>
+          <t>-9.76%</t>
         </is>
       </c>
     </row>
@@ -791,32 +791,32 @@
       </c>
       <c r="B10" s="18" t="inlineStr">
         <is>
-          <t>17.90%</t>
+          <t>17.81%</t>
         </is>
       </c>
       <c r="C10" s="18" t="inlineStr">
         <is>
-          <t>15.16%</t>
+          <t>15.07%</t>
         </is>
       </c>
       <c r="D10" s="18" t="inlineStr">
         <is>
-          <t>15.67%</t>
+          <t>15.59%</t>
         </is>
       </c>
       <c r="E10" s="18" t="inlineStr">
         <is>
-          <t>-12.02%</t>
+          <t>-11.98%</t>
         </is>
       </c>
       <c r="F10" s="18" t="inlineStr">
         <is>
-          <t>13.41%</t>
+          <t>13.38%</t>
         </is>
       </c>
       <c r="G10" s="19" t="inlineStr">
         <is>
-          <t>-10.96%</t>
+          <t>-11.02%</t>
         </is>
       </c>
     </row>
@@ -828,32 +828,32 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>16.91%</t>
+          <t>16.99%</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>16.80%</t>
+          <t>17.11%</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
-          <t>17.87%</t>
+          <t>17.93%</t>
         </is>
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>21.34%</t>
+          <t>21.37%</t>
         </is>
       </c>
       <c r="F11" s="12" t="inlineStr">
         <is>
-          <t>16.86%</t>
+          <t>17.04%</t>
         </is>
       </c>
       <c r="G11" s="13" t="inlineStr">
         <is>
-          <t>19.43%</t>
+          <t>19.32%</t>
         </is>
       </c>
     </row>
@@ -865,17 +865,17 @@
       </c>
       <c r="B12" s="18" t="inlineStr">
         <is>
-          <t>1.07</t>
+          <t>1.06</t>
         </is>
       </c>
       <c r="C12" s="18" t="inlineStr">
         <is>
-          <t>0.93</t>
+          <t>0.91</t>
         </is>
       </c>
       <c r="D12" s="18" t="inlineStr">
         <is>
-          <t>0.91</t>
+          <t>0.90</t>
         </is>
       </c>
       <c r="E12" s="18" t="inlineStr">
@@ -890,7 +890,7 @@
       </c>
       <c r="G12" s="19" t="inlineStr">
         <is>
-          <t>-0.50</t>
+          <t>-0.51</t>
         </is>
       </c>
     </row>
@@ -902,32 +902,32 @@
       </c>
       <c r="B13" s="21" t="inlineStr">
         <is>
-          <t>-37.98%</t>
+          <t>-39.28%</t>
         </is>
       </c>
       <c r="C13" s="21" t="inlineStr">
         <is>
-          <t>-46.48%</t>
+          <t>-44.95%</t>
         </is>
       </c>
       <c r="D13" s="21" t="inlineStr">
         <is>
-          <t>-46.06%</t>
+          <t>-46.86%</t>
         </is>
       </c>
       <c r="E13" s="21" t="inlineStr">
         <is>
-          <t>-99.83%</t>
+          <t>-99.82%</t>
         </is>
       </c>
       <c r="F13" s="21" t="inlineStr">
         <is>
-          <t>-47.56%</t>
+          <t>-46.72%</t>
         </is>
       </c>
       <c r="G13" s="22" t="inlineStr">
         <is>
-          <t>-99.67%</t>
+          <t>-99.68%</t>
         </is>
       </c>
     </row>
@@ -946,17 +946,17 @@
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>1.82</t>
+          <t>1.80</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>1.59</t>
+          <t>1.54</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
         <is>
-          <t>1.51</t>
+          <t>1.50</t>
         </is>
       </c>
       <c r="E15" s="12" t="inlineStr">
@@ -966,7 +966,7 @@
       </c>
       <c r="F15" s="12" t="inlineStr">
         <is>
-          <t>1.37</t>
+          <t>1.35</t>
         </is>
       </c>
       <c r="G15" s="13" t="inlineStr">
@@ -983,12 +983,12 @@
       </c>
       <c r="B16" s="18" t="inlineStr">
         <is>
-          <t>0.47</t>
+          <t>0.46</t>
         </is>
       </c>
       <c r="C16" s="18" t="inlineStr">
         <is>
-          <t>0.34</t>
+          <t>0.35</t>
         </is>
       </c>
       <c r="D16" s="18" t="inlineStr">
@@ -1057,32 +1057,32 @@
       </c>
       <c r="B18" s="18" t="inlineStr">
         <is>
-          <t>64.9%</t>
+          <t>64.7%</t>
         </is>
       </c>
       <c r="C18" s="18" t="inlineStr">
         <is>
-          <t>62.0%</t>
+          <t>61.5%</t>
         </is>
       </c>
       <c r="D18" s="18" t="inlineStr">
         <is>
-          <t>62.4%</t>
+          <t>63.0%</t>
         </is>
       </c>
       <c r="E18" s="18" t="inlineStr">
         <is>
-          <t>40.4%</t>
+          <t>40.5%</t>
         </is>
       </c>
       <c r="F18" s="18" t="inlineStr">
         <is>
-          <t>61.9%</t>
+          <t>61.7%</t>
         </is>
       </c>
       <c r="G18" s="19" t="inlineStr">
         <is>
-          <t>39.7%</t>
+          <t>40.2%</t>
         </is>
       </c>
     </row>
@@ -1099,7 +1099,7 @@
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>-0.08</t>
+          <t>-0.10</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
@@ -1109,17 +1109,17 @@
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>0.61</t>
+          <t>0.59</t>
         </is>
       </c>
       <c r="F19" s="12" t="inlineStr">
         <is>
-          <t>-0.19</t>
+          <t>-0.20</t>
         </is>
       </c>
       <c r="G19" s="13" t="inlineStr">
         <is>
-          <t>0.54</t>
+          <t>0.53</t>
         </is>
       </c>
     </row>
@@ -1131,32 +1131,32 @@
       </c>
       <c r="B20" s="15" t="inlineStr">
         <is>
-          <t>1.76</t>
+          <t>1.77</t>
         </is>
       </c>
       <c r="C20" s="15" t="inlineStr">
         <is>
-          <t>1.66</t>
+          <t>1.80</t>
         </is>
       </c>
       <c r="D20" s="15" t="inlineStr">
         <is>
-          <t>2.29</t>
+          <t>2.28</t>
         </is>
       </c>
       <c r="E20" s="15" t="inlineStr">
         <is>
-          <t>2.73</t>
+          <t>2.65</t>
         </is>
       </c>
       <c r="F20" s="15" t="inlineStr">
         <is>
-          <t>1.81</t>
+          <t>1.91</t>
         </is>
       </c>
       <c r="G20" s="16" t="inlineStr">
         <is>
-          <t>2.79</t>
+          <t>2.75</t>
         </is>
       </c>
     </row>
@@ -1175,32 +1175,32 @@
       </c>
       <c r="B22" s="12" t="inlineStr">
         <is>
-          <t>7.45</t>
+          <t>7.39</t>
         </is>
       </c>
       <c r="C22" s="12" t="inlineStr">
         <is>
-          <t>6.49</t>
+          <t>6.37</t>
         </is>
       </c>
       <c r="D22" s="12" t="inlineStr">
         <is>
-          <t>6.46</t>
+          <t>6.42</t>
         </is>
       </c>
       <c r="E22" s="12" t="inlineStr">
         <is>
-          <t>-3.43</t>
+          <t>-3.41</t>
         </is>
       </c>
       <c r="F22" s="12" t="inlineStr">
         <is>
-          <t>5.93</t>
+          <t>5.87</t>
         </is>
       </c>
       <c r="G22" s="13" t="inlineStr">
         <is>
-          <t>-3.48</t>
+          <t>-3.53</t>
         </is>
       </c>
     </row>
@@ -1227,7 +1227,7 @@
       </c>
       <c r="E23" s="18" t="inlineStr">
         <is>
-          <t>0.0006</t>
+          <t>0.0007</t>
         </is>
       </c>
       <c r="F23" s="18" t="inlineStr">
@@ -1237,7 +1237,7 @@
       </c>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>0.0005</t>
+          <t>0.0004</t>
         </is>
       </c>
     </row>
@@ -1249,32 +1249,32 @@
       </c>
       <c r="B24" s="21" t="inlineStr">
         <is>
-          <t>[13.27%, 22.75%]</t>
+          <t>[13.19%, 22.71%]</t>
         </is>
       </c>
       <c r="C24" s="21" t="inlineStr">
         <is>
-          <t>[10.89%, 20.31%]</t>
+          <t>[10.78%, 20.37%]</t>
         </is>
       </c>
       <c r="D24" s="21" t="inlineStr">
         <is>
-          <t>[11.31%, 21.17%]</t>
+          <t>[11.24%, 21.13%]</t>
         </is>
       </c>
       <c r="E24" s="21" t="inlineStr">
         <is>
-          <t>[-16.46%, -4.50%]</t>
+          <t>[-16.42%, -4.44%]</t>
         </is>
       </c>
       <c r="F24" s="21" t="inlineStr">
         <is>
-          <t>[9.42%, 18.72%]</t>
+          <t>[9.37%, 18.77%]</t>
         </is>
       </c>
       <c r="G24" s="22" t="inlineStr">
         <is>
-          <t>[-15.12%, -4.23%]</t>
+          <t>[-15.17%, -4.35%]</t>
         </is>
       </c>
     </row>
@@ -1293,32 +1293,32 @@
       </c>
       <c r="B26" s="12" t="inlineStr">
         <is>
-          <t>5.60%</t>
+          <t>5.50%</t>
         </is>
       </c>
       <c r="C26" s="12" t="inlineStr">
         <is>
-          <t>4.02%</t>
+          <t>3.89%</t>
         </is>
       </c>
       <c r="D26" s="12" t="inlineStr">
         <is>
-          <t>3.22%</t>
+          <t>3.15%</t>
         </is>
       </c>
       <c r="E26" s="12" t="inlineStr">
         <is>
-          <t>0.16%</t>
+          <t>0.17%</t>
         </is>
       </c>
       <c r="F26" s="12" t="inlineStr">
         <is>
-          <t>1.79%</t>
+          <t>1.73%</t>
         </is>
       </c>
       <c r="G26" s="13" t="inlineStr">
         <is>
-          <t>-0.02%</t>
+          <t>-0.16%</t>
         </is>
       </c>
     </row>
@@ -1330,32 +1330,32 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
+          <t>1.11%</t>
+        </is>
+      </c>
+      <c r="C27" s="18" t="inlineStr">
+        <is>
+          <t>1.58%</t>
+        </is>
+      </c>
+      <c r="D27" s="18" t="inlineStr">
+        <is>
+          <t>0.89%</t>
+        </is>
+      </c>
+      <c r="E27" s="18" t="inlineStr">
+        <is>
+          <t>1.27%</t>
+        </is>
+      </c>
+      <c r="F27" s="18" t="inlineStr">
+        <is>
           <t>1.09%</t>
         </is>
       </c>
-      <c r="C27" s="18" t="inlineStr">
-        <is>
-          <t>1.54%</t>
-        </is>
-      </c>
-      <c r="D27" s="18" t="inlineStr">
-        <is>
-          <t>0.86%</t>
-        </is>
-      </c>
-      <c r="E27" s="18" t="inlineStr">
-        <is>
-          <t>1.25%</t>
-        </is>
-      </c>
-      <c r="F27" s="18" t="inlineStr">
-        <is>
-          <t>1.07%</t>
-        </is>
-      </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>1.28%</t>
+          <t>1.24%</t>
         </is>
       </c>
     </row>
@@ -1367,17 +1367,17 @@
       </c>
       <c r="B28" s="12" t="inlineStr">
         <is>
-          <t>5.14</t>
+          <t>4.96</t>
         </is>
       </c>
       <c r="C28" s="12" t="inlineStr">
         <is>
-          <t>2.60</t>
+          <t>2.47</t>
         </is>
       </c>
       <c r="D28" s="12" t="inlineStr">
         <is>
-          <t>3.73</t>
+          <t>3.53</t>
         </is>
       </c>
       <c r="E28" s="12" t="inlineStr">
@@ -1387,12 +1387,12 @@
       </c>
       <c r="F28" s="12" t="inlineStr">
         <is>
-          <t>1.67</t>
+          <t>1.58</t>
         </is>
       </c>
       <c r="G28" s="13" t="inlineStr">
         <is>
-          <t>-0.01</t>
+          <t>-0.13</t>
         </is>
       </c>
     </row>
@@ -1409,27 +1409,27 @@
       </c>
       <c r="C29" s="18" t="inlineStr">
         <is>
-          <t>0.0092</t>
+          <t>0.0135</t>
         </is>
       </c>
       <c r="D29" s="18" t="inlineStr">
         <is>
-          <t>0.0002</t>
+          <t>0.0004</t>
         </is>
       </c>
       <c r="E29" s="18" t="inlineStr">
         <is>
-          <t>0.8968</t>
+          <t>0.8942</t>
         </is>
       </c>
       <c r="F29" s="18" t="inlineStr">
         <is>
-          <t>0.0950</t>
+          <t>0.1135</t>
         </is>
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>0.9905</t>
+          <t>0.8961</t>
         </is>
       </c>
     </row>
@@ -1441,32 +1441,32 @@
       </c>
       <c r="B30" s="12" t="inlineStr">
         <is>
-          <t>[3.46%, 7.73%]</t>
+          <t>[3.32%, 7.67%]</t>
         </is>
       </c>
       <c r="C30" s="12" t="inlineStr">
         <is>
-          <t>[1.00%, 7.05%]</t>
+          <t>[0.81%, 6.98%]</t>
         </is>
       </c>
       <c r="D30" s="12" t="inlineStr">
         <is>
-          <t>[1.53%, 4.92%]</t>
+          <t>[1.40%, 4.89%]</t>
         </is>
       </c>
       <c r="E30" s="12" t="inlineStr">
         <is>
-          <t>[-2.28%, 2.60%]</t>
+          <t>[-2.32%, 2.66%]</t>
         </is>
       </c>
       <c r="F30" s="12" t="inlineStr">
         <is>
-          <t>[-0.31%, 3.89%]</t>
+          <t>[-0.41%, 3.87%]</t>
         </is>
       </c>
       <c r="G30" s="13" t="inlineStr">
         <is>
-          <t>[-2.51%, 2.48%]</t>
+          <t>[-2.59%, 2.27%]</t>
         </is>
       </c>
     </row>
@@ -1478,32 +1478,32 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>0.990</t>
+          <t>0.995</t>
         </is>
       </c>
       <c r="C31" s="18" t="inlineStr">
         <is>
-          <t>0.889</t>
+          <t>0.902</t>
         </is>
       </c>
       <c r="D31" s="18" t="inlineStr">
         <is>
-          <t>1.038</t>
+          <t>1.040</t>
         </is>
       </c>
       <c r="E31" s="18" t="inlineStr">
         <is>
-          <t>-1.279</t>
+          <t>-1.274</t>
         </is>
       </c>
       <c r="F31" s="18" t="inlineStr">
         <is>
-          <t>0.951</t>
+          <t>0.958</t>
         </is>
       </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>-1.161</t>
+          <t>-1.154</t>
         </is>
       </c>
     </row>
@@ -1515,32 +1515,32 @@
       </c>
       <c r="B32" s="21" t="inlineStr">
         <is>
-          <t>39.22</t>
+          <t>39.75</t>
         </is>
       </c>
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>19.58</t>
+          <t>19.27</t>
         </is>
       </c>
       <c r="D32" s="21" t="inlineStr">
         <is>
-          <t>37.12</t>
+          <t>37.44</t>
         </is>
       </c>
       <c r="E32" s="21" t="inlineStr">
         <is>
-          <t>-39.61</t>
+          <t>-39.62</t>
         </is>
       </c>
       <c r="F32" s="21" t="inlineStr">
         <is>
-          <t>32.26</t>
+          <t>30.89</t>
         </is>
       </c>
       <c r="G32" s="22" t="inlineStr">
         <is>
-          <t>-31.25</t>
+          <t>-34.65</t>
         </is>
       </c>
     </row>

</xml_diff>